<commit_message>
Update stringybark data and rename CSV files
</commit_message>
<xml_diff>
--- a/Stringybark/stringybark.xlsx
+++ b/Stringybark/stringybark.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud-my.sharepoint.com/personal/haninhn_student_unimelb_edu_au/Documents/Documents/Chapter 2/Chapter 2 data/Stringybark/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="301" documentId="11_F25DC773A252ABDACC10487769DB591E5BDE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90CD098F-B1E8-E04E-BC36-94273EC60BB1}"/>
+  <xr:revisionPtr revIDLastSave="302" documentId="11_F25DC773A252ABDACC10487769DB591E5BDE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EDC16ADB-BC29-2345-AFD0-F79169D5D2D7}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-13900" windowWidth="38400" windowHeight="21000" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-5860" windowWidth="38400" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="E  obliqua 90% char T17" sheetId="11" r:id="rId1"/>
@@ -352,7 +352,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4354" uniqueCount="1239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4354" uniqueCount="1240">
   <si>
     <t>Source.Name</t>
   </si>
@@ -4069,6 +4069,9 @@
   </si>
   <si>
     <t>Density (kg/m3)</t>
+  </si>
+  <si>
+    <t>S12b.csv</t>
   </si>
 </sst>
 </file>
@@ -4110,10 +4113,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -4155,10 +4155,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4255,8 +4251,8 @@
     <sortCondition ref="C1:C302"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{5B3B79D8-C44A-4716-85F8-54B8B21843E6}" uniqueName="1" name="Source.Name" queryTableFieldId="1" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{FBD25F70-8F20-4880-BD44-67149364EF17}" uniqueName="2" name="File (ID)" queryTableFieldId="2" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{5B3B79D8-C44A-4716-85F8-54B8B21843E6}" uniqueName="1" name="Source.Name" queryTableFieldId="1" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{FBD25F70-8F20-4880-BD44-67149364EF17}" uniqueName="2" name="File (ID)" queryTableFieldId="2" dataDxfId="6"/>
     <tableColumn id="3" xr3:uid="{807F55D5-B2CA-49C8-BC1E-D84D0F756901}" uniqueName="3" name="Volume (mm3)" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{0818186D-F74B-4BA5-826E-6099407249A3}" uniqueName="4" name="Surface Area (mm2)" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{32C8C197-2582-46CB-BFA0-DAB87A90C99B}" uniqueName="5" name="Length (mm)" queryTableFieldId="5"/>
@@ -4275,8 +4271,8 @@
     <sortCondition ref="C1:C204"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{B3C7DBA4-D3D1-4B12-91B2-23153CBD04B0}" uniqueName="1" name="Source.Name" queryTableFieldId="1" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{4A058920-EFE5-4AF6-972E-7D2F6882EEF9}" uniqueName="2" name="File (ID)" queryTableFieldId="2" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{B3C7DBA4-D3D1-4B12-91B2-23153CBD04B0}" uniqueName="1" name="Source.Name" queryTableFieldId="1"/>
+    <tableColumn id="2" xr3:uid="{4A058920-EFE5-4AF6-972E-7D2F6882EEF9}" uniqueName="2" name="File (ID)" queryTableFieldId="2" dataDxfId="5"/>
     <tableColumn id="3" xr3:uid="{1A06E7E1-C8F4-46D1-A293-343B73231FD1}" uniqueName="3" name="Volume (mm3)" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{30CA3A4B-E501-4AF1-AA66-2C804763CC5C}" uniqueName="4" name="Surface Area (mm2)" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{3E1C8902-EAB2-493E-8B89-C8BD536BC79A}" uniqueName="5" name="Length (mm)" queryTableFieldId="5"/>
@@ -4295,8 +4291,8 @@
     <sortCondition ref="C1:C697"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{1BA4FC3A-493C-49B1-81B8-DCF6364F871A}" uniqueName="1" name="Source.Name" queryTableFieldId="1" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{37ACD0C7-839E-46F5-ADF7-3F6D404CE1C1}" uniqueName="2" name="File (ID)" queryTableFieldId="2" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{1BA4FC3A-493C-49B1-81B8-DCF6364F871A}" uniqueName="1" name="Source.Name" queryTableFieldId="1" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{37ACD0C7-839E-46F5-ADF7-3F6D404CE1C1}" uniqueName="2" name="File (ID)" queryTableFieldId="2" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{380AD657-E7AF-4698-882D-DD4ABD7E38D8}" uniqueName="3" name="Volume (mm3)" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{3627BC35-1CAE-4359-A63D-F893914B4794}" uniqueName="4" name="Surface Area (mm2)" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{742BE2C1-E138-4EBA-9742-0F94ECF814EA}" uniqueName="5" name="Length (mm)" queryTableFieldId="5"/>
@@ -4315,15 +4311,15 @@
     <sortCondition descending="1" ref="I1:I323"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{AB5E7E98-A7E2-452B-A5E0-F71C30E90EA5}" uniqueName="1" name="Source.Name" queryTableFieldId="1" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{23576739-D5C3-4BEC-84C5-C81FFFBB3B36}" uniqueName="2" name="File (ID)" queryTableFieldId="2" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{AB5E7E98-A7E2-452B-A5E0-F71C30E90EA5}" uniqueName="1" name="Source.Name" queryTableFieldId="1" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{23576739-D5C3-4BEC-84C5-C81FFFBB3B36}" uniqueName="2" name="File (ID)" queryTableFieldId="2" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{D45212C2-6966-4DEB-87CE-7E4064EFE434}" uniqueName="3" name="Volume (mm3)" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{EFCD693F-4240-4AB6-819B-3B801ABF557A}" uniqueName="4" name="Surface Area (mm2)" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{5584ECA4-D1AD-4750-9820-A8CB3615B575}" uniqueName="5" name="Length (mm)" queryTableFieldId="5"/>
     <tableColumn id="6" xr3:uid="{C8496460-E683-42A5-A266-BEC35F8EC4D6}" uniqueName="6" name="Width (mm)" queryTableFieldId="6"/>
     <tableColumn id="7" xr3:uid="{13A3098C-A238-4CE6-BEE9-15B24F5F9D0F}" uniqueName="7" name="Height (mm)" queryTableFieldId="7"/>
     <tableColumn id="8" xr3:uid="{3EE15122-99B8-4FD7-AC43-7840B4992BF1}" uniqueName="8" name="Mass (g)" queryTableFieldId="8"/>
-    <tableColumn id="9" xr3:uid="{9D00BC0A-D4A2-AA45-A2E5-2059B40B0E30}" uniqueName="9" name="Density (kg/m3)" queryTableFieldId="9" dataDxfId="2">
+    <tableColumn id="9" xr3:uid="{9D00BC0A-D4A2-AA45-A2E5-2059B40B0E30}" uniqueName="9" name="Density (kg/m3)" queryTableFieldId="9" dataDxfId="0">
       <calculatedColumnFormula>E__obliqua_0__char_T5__3[[#This Row],[Mass (g)]]/E__obliqua_0__char_T5__3[[#This Row],[Volume (mm3)]]*1000000</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4338,8 +4334,8 @@
     <sortCondition descending="1" ref="I1:I35"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{DFD6DDC3-8515-4D61-B02A-40FD4FF9059F}" uniqueName="1" name="Source.Name" queryTableFieldId="1" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{3199625E-6D42-429C-A444-8187A5B89797}" uniqueName="2" name="File (ID)" queryTableFieldId="2" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{DFD6DDC3-8515-4D61-B02A-40FD4FF9059F}" uniqueName="1" name="Source.Name" queryTableFieldId="1" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{3199625E-6D42-429C-A444-8187A5B89797}" uniqueName="2" name="File (ID)" queryTableFieldId="2" dataDxfId="8"/>
     <tableColumn id="3" xr3:uid="{43BBAFDD-411A-45A3-B08A-C0552BC1D9DD}" uniqueName="3" name="Volume (mm3)" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{ECE74D4E-248C-49EE-B777-D3624919B7B0}" uniqueName="4" name="Surface Area (mm2)" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{DDF6C964-B51D-4D51-A171-545522DB5918}" uniqueName="5" name="Length (mm)" queryTableFieldId="5"/>
@@ -12531,7 +12527,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>1024</v>
+        <v>94</v>
       </c>
       <c r="B2" t="s">
         <v>1026</v>
@@ -12661,7 +12657,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>1024</v>
+        <v>94</v>
       </c>
       <c r="B7" t="s">
         <v>516</v>
@@ -12739,7 +12735,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>1024</v>
+        <v>94</v>
       </c>
       <c r="B10" t="s">
         <v>96</v>
@@ -13259,7 +13255,7 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>1024</v>
+        <v>94</v>
       </c>
       <c r="B30" t="s">
         <v>1025</v>
@@ -14013,7 +14009,7 @@
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>1024</v>
+        <v>94</v>
       </c>
       <c r="B59" t="s">
         <v>95</v>
@@ -14429,7 +14425,7 @@
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>1024</v>
+        <v>94</v>
       </c>
       <c r="B75" t="s">
         <v>517</v>
@@ -14767,7 +14763,7 @@
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>34</v>
+        <v>1239</v>
       </c>
       <c r="B88" t="s">
         <v>997</v>
@@ -15677,7 +15673,7 @@
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>1024</v>
+        <v>94</v>
       </c>
       <c r="B123" t="s">
         <v>515</v>
@@ -16119,7 +16115,7 @@
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
-        <v>34</v>
+        <v>1239</v>
       </c>
       <c r="B140" t="s">
         <v>996</v>
@@ -16379,7 +16375,7 @@
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
-        <v>1024</v>
+        <v>94</v>
       </c>
       <c r="B150" t="s">
         <v>97</v>

</xml_diff>